<commit_message>
Updated LVA model - 2025-11-06 15:20
</commit_message>
<xml_diff>
--- a/VerveStacks_LVA/SubRES_Tmpl/SubRES_New_RE_and_Conventional.xlsx
+++ b/VerveStacks_LVA/SubRES_Tmpl/SubRES_New_RE_and_Conventional.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Veda\Veda\Veda_models\vervestacks_models\VerveStacks_LVA\SubRES_Tmpl\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{749BCECA-687B-4870-8507-91704E06EA01}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{6493F9C8-F642-44E5-A948-924426A14006}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" firstSheet="6" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -5715,7 +5715,7 @@
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{038EC51F-5DD8-4170-87CE-CBBF6F8C2156}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5F3638AA-B23C-4093-ADC4-707C833E9EAC}">
   <dimension ref="B9:M20"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -6118,7 +6118,7 @@
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EED4F4BF-4E1A-4BFF-9C8F-8E917A20E02A}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EC8FB6AD-BCE3-41D4-B8C5-749FE7994A83}">
   <dimension ref="B9:Z20"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -6890,7 +6890,7 @@
 </file>
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4CF9E94A-1A5E-40F0-B942-3B039316A77B}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3BD6F30F-AF66-4A16-A53F-5214B3D995CF}">
   <dimension ref="B9:P73"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>

</xml_diff>

<commit_message>
Updated LVA model - 2025-11-06 15:41
</commit_message>
<xml_diff>
--- a/VerveStacks_LVA/SubRES_Tmpl/SubRES_New_RE_and_Conventional.xlsx
+++ b/VerveStacks_LVA/SubRES_Tmpl/SubRES_New_RE_and_Conventional.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Veda\Veda\Veda_models\vervestacks_models\VerveStacks_LVA\SubRES_Tmpl\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{6493F9C8-F642-44E5-A948-924426A14006}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{160EBBA3-F2E5-426A-A8C6-E111917C9924}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" firstSheet="6" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -5715,7 +5715,7 @@
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5F3638AA-B23C-4093-ADC4-707C833E9EAC}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{75E619C6-B40B-43CE-95D9-FFBE7B34E73C}">
   <dimension ref="B9:M20"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -6118,7 +6118,7 @@
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EC8FB6AD-BCE3-41D4-B8C5-749FE7994A83}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6183695B-3B6B-4B30-BB0D-DB5B5B290A67}">
   <dimension ref="B9:Z20"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -6890,7 +6890,7 @@
 </file>
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3BD6F30F-AF66-4A16-A53F-5214B3D995CF}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BB580C7C-6034-4888-8333-F56B813ED2CC}">
   <dimension ref="B9:P73"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>

</xml_diff>

<commit_message>
Updated LVA model - 2025-11-06 15:50
</commit_message>
<xml_diff>
--- a/VerveStacks_LVA/SubRES_Tmpl/SubRES_New_RE_and_Conventional.xlsx
+++ b/VerveStacks_LVA/SubRES_Tmpl/SubRES_New_RE_and_Conventional.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Veda\Veda\Veda_models\vervestacks_models\VerveStacks_LVA\SubRES_Tmpl\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{160EBBA3-F2E5-426A-A8C6-E111917C9924}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{AD656EA4-0E8C-42B1-92D4-2EA2C9D840EC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" firstSheet="6" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -5715,7 +5715,7 @@
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{75E619C6-B40B-43CE-95D9-FFBE7B34E73C}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{52EB6F4E-B724-499F-9FD3-D6B974818D35}">
   <dimension ref="B9:M20"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -6118,7 +6118,7 @@
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6183695B-3B6B-4B30-BB0D-DB5B5B290A67}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4F92782F-6648-4D1F-B85E-92857A355026}">
   <dimension ref="B9:Z20"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -6890,7 +6890,7 @@
 </file>
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BB580C7C-6034-4888-8333-F56B813ED2CC}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{171BBAA6-6D3E-46FF-B1C9-38600B192ECE}">
   <dimension ref="B9:P73"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>

</xml_diff>

<commit_message>
Updated LVA model - 2025-11-06 15:57
</commit_message>
<xml_diff>
--- a/VerveStacks_LVA/SubRES_Tmpl/SubRES_New_RE_and_Conventional.xlsx
+++ b/VerveStacks_LVA/SubRES_Tmpl/SubRES_New_RE_and_Conventional.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Veda\Veda\Veda_models\vervestacks_models\VerveStacks_LVA\SubRES_Tmpl\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{AD656EA4-0E8C-42B1-92D4-2EA2C9D840EC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{68BBB301-0C26-42E1-A568-2D9FBDB131B0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" firstSheet="6" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -5715,7 +5715,7 @@
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{52EB6F4E-B724-499F-9FD3-D6B974818D35}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{801B390C-F793-46A0-8F4E-8862A4836DD5}">
   <dimension ref="B9:M20"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -6118,7 +6118,7 @@
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4F92782F-6648-4D1F-B85E-92857A355026}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E00ABDA5-083F-4DBC-9EBA-C03F90B82FD9}">
   <dimension ref="B9:Z20"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -6890,7 +6890,7 @@
 </file>
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{171BBAA6-6D3E-46FF-B1C9-38600B192ECE}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BBD36140-4A19-4941-97BE-5DA2327AE4CE}">
   <dimension ref="B9:P73"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>

</xml_diff>

<commit_message>
Updated LVA model - 2025-11-06 16:00
</commit_message>
<xml_diff>
--- a/VerveStacks_LVA/SubRES_Tmpl/SubRES_New_RE_and_Conventional.xlsx
+++ b/VerveStacks_LVA/SubRES_Tmpl/SubRES_New_RE_and_Conventional.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Veda\Veda\Veda_models\vervestacks_models\VerveStacks_LVA\SubRES_Tmpl\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{68BBB301-0C26-42E1-A568-2D9FBDB131B0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{5B47CB1A-45AE-4B8B-8E42-5635CAC4CF55}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" firstSheet="6" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -5715,7 +5715,7 @@
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{801B390C-F793-46A0-8F4E-8862A4836DD5}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{56A294DB-8E37-4E63-AF1D-BC43E7839402}">
   <dimension ref="B9:M20"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -6118,7 +6118,7 @@
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E00ABDA5-083F-4DBC-9EBA-C03F90B82FD9}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{927656FD-F3A8-4609-A154-C141F15F29F5}">
   <dimension ref="B9:Z20"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -6890,7 +6890,7 @@
 </file>
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BBD36140-4A19-4941-97BE-5DA2327AE4CE}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2203839B-7588-4571-A146-9D179A1E20C6}">
   <dimension ref="B9:P73"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>

</xml_diff>

<commit_message>
Updated LVA model - 2025-11-06 16:05
</commit_message>
<xml_diff>
--- a/VerveStacks_LVA/SubRES_Tmpl/SubRES_New_RE_and_Conventional.xlsx
+++ b/VerveStacks_LVA/SubRES_Tmpl/SubRES_New_RE_and_Conventional.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Veda\Veda\Veda_models\vervestacks_models\VerveStacks_LVA\SubRES_Tmpl\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{5B47CB1A-45AE-4B8B-8E42-5635CAC4CF55}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{F4476EA7-99A1-4ACF-9206-9C3F71AB9CA1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" firstSheet="6" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -5715,7 +5715,7 @@
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{56A294DB-8E37-4E63-AF1D-BC43E7839402}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BF509289-BCD8-4C4A-83B4-DD1193862AFD}">
   <dimension ref="B9:M20"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -6118,7 +6118,7 @@
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{927656FD-F3A8-4609-A154-C141F15F29F5}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3ED954A0-34F0-4284-8769-3B6A6CD6890A}">
   <dimension ref="B9:Z20"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -6890,7 +6890,7 @@
 </file>
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2203839B-7588-4571-A146-9D179A1E20C6}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{60ACF7A6-2B8B-4A7D-A5CA-DDC16C861F9D}">
   <dimension ref="B9:P73"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>

</xml_diff>